<commit_message>
feat(deploy): configure and harden production subdomain erp.arivahly.in and update control-plane registry
</commit_message>
<xml_diff>
--- a/docs/control-plane/00_MASTER_CONTROL_INDEX.xlsx
+++ b/docs/control-plane/00_MASTER_CONTROL_INDEX.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="293">
   <si>
     <t>00_MASTER_CONTROL_INDEX</t>
   </si>
@@ -48,6 +48,12 @@
     <t>CRITICAL: NEVER STORE PASSWORDS, API KEYS, SERVICE-ROLE KEYS, PRIVATE CERTIFICATES, SMTP PASSWORDS, OR R2 SECRETS IN THIS WORKBOOK. USE SECURE ENVIRONMENT REFERENCES ONLY.</t>
   </si>
   <si>
+    <t>Canonical Production Subdomain</t>
+  </si>
+  <si>
+    <t>https://erp.arivahly.in (Parent domain: arivahly.in)</t>
+  </si>
+  <si>
     <t>AI Operating Constraint 1</t>
   </si>
   <si>
@@ -72,10 +78,16 @@
     <t>UNKNOWN means unknown. Do not guess. If a field is uncertain, record NEEDS_VERIFICATION.</t>
   </si>
   <si>
+    <t>MCP Security Boundary</t>
+  </si>
+  <si>
+    <t>MCP is DISABLED and BLOCKED from public routing. MCP tools must remain internal/local only.</t>
+  </si>
+  <si>
     <t>Last Audit Date</t>
   </si>
   <si>
-    <t>2026-09-05T13:10:00+05:30 (Release v1.1.2-online-production-hardened)</t>
+    <t>2026-09-05T13:20:00+05:30 (Release v1.1.2-online-production-hardened)</t>
   </si>
   <si>
     <t>Record_ID</t>
@@ -297,7 +309,7 @@
     <t>ONLINE_PROD</t>
   </si>
   <si>
-    <t>maatarajewellers.shop under Cloudflare Full (Strict) SSL</t>
+    <t>erp.arivahly.in under Cloudflare Full (Strict) SSL</t>
   </si>
   <si>
     <t>CTRL-011</t>
@@ -540,13 +552,13 @@
     <t>DOM-&lt;HOSTNAME&gt;-&lt;ENV&gt;</t>
   </si>
   <si>
-    <t>DOM-MAATARA-PROD</t>
+    <t>DOM-ARIVAHLY-ERP</t>
   </si>
   <si>
     <t>Fully qualified domain record</t>
   </si>
   <si>
-    <t>Maps to Cloudflare zone and origin host</t>
+    <t>Maps to Cloudflare zone and origin host (e.g. erp.arivahly.in)</t>
   </si>
   <si>
     <t>Service ID</t>
@@ -606,15 +618,21 @@
     <t>Severity</t>
   </si>
   <si>
+    <t>Canonical Domain</t>
+  </si>
+  <si>
+    <t>Production Online Managed ERP URL is strictly https://erp.arivahly.in. Never deploy to root domain or temporary hosts.</t>
+  </si>
+  <si>
+    <t>CRITICAL</t>
+  </si>
+  <si>
     <t>No Account Inference</t>
   </si>
   <si>
     <t>Never infer account relationships from similar names. Always verify explicit Account_ID.</t>
   </si>
   <si>
-    <t>CRITICAL</t>
-  </si>
-  <si>
     <t>Distinct Accounts</t>
   </si>
   <si>
@@ -660,16 +678,10 @@
     <t>Never assume R2 buckets belong to the same environment. Keys must remain strictly tenant-scoped.</t>
   </si>
   <si>
-    <t>No Config Copying</t>
-  </si>
-  <si>
-    <t>Never copy production configuration into another environment without explicit user authorization.</t>
-  </si>
-  <si>
-    <t>No Cross-Env Secrets</t>
-  </si>
-  <si>
-    <t>Never use a secret or key from another environment. Stored in secure host envs only.</t>
+    <t>MCP Public Route Block</t>
+  </si>
+  <si>
+    <t>MCP tools must remain disabled/blocked from public network routing.</t>
   </si>
   <si>
     <t>Resolution Hierarchy</t>
@@ -828,7 +840,7 @@
     <t>Total Domains Configured</t>
   </si>
   <si>
-    <t>maatarajewellers.shop, www.maatarajewellers.shop</t>
+    <t>erp.arivahly.in (Subdomain), arivahly.in (Parent Root)</t>
   </si>
   <si>
     <t>Total Backend Services</t>
@@ -864,10 +876,19 @@
     <t>Future MCP Endpoint intentionally BLOCKED/DISABLED per security directive</t>
   </si>
   <si>
+    <t>Canonical Production URL</t>
+  </si>
+  <si>
+    <t>https://erp.arivahly.in</t>
+  </si>
+  <si>
+    <t>Official human-facing production URL</t>
+  </si>
+  <si>
     <t>Overall Verification Timestamp</t>
   </si>
   <si>
-    <t>2026-09-05T13:10:00+05:30</t>
+    <t>2026-09-05T13:20:00+05:30</t>
   </si>
   <si>
     <t>FINAL_ONLINE_PRODUCTION_AUDIT.md</t>
@@ -1321,7 +1342,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1406,6 +1427,22 @@
       </c>
       <c r="B11" s="4" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1434,737 +1471,737 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="I3" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="6" t="s">
+      <c r="J3" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>39</v>
-      </c>
       <c r="K3" s="6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D6" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>57</v>
-      </c>
       <c r="G6" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>50</v>
-      </c>
       <c r="G7" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D9" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="G9" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D12" s="6" t="s">
+      <c r="G12" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="E12" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>92</v>
-      </c>
       <c r="H12" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>112</v>
-      </c>
       <c r="D16" s="6" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>133</v>
-      </c>
       <c r="D20" s="6" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -2187,155 +2224,155 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -2357,16 +2394,16 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2374,13 +2411,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2388,13 +2425,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2402,13 +2439,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>202</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2416,13 +2453,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2430,13 +2467,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2444,13 +2481,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2458,13 +2495,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2472,13 +2509,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2486,13 +2523,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2500,13 +2537,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2514,13 +2551,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -2552,190 +2589,190 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="N2" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2746,7 +2783,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -2757,156 +2794,170 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B2" s="6">
         <v>6</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B3" s="6">
         <v>3</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="B4" s="6">
         <v>3</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B5" s="6">
         <v>2</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B6" s="6">
         <v>7</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="B7" s="6">
         <v>3</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="B8" s="6">
         <v>1</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B9" s="6">
         <v>0</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B10" s="6">
         <v>1</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>284</v>
+        <v>92</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>285</v>
+        <v>288</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(control-plane): document strict dual-track ownership for Public Website vs Online ERP
</commit_message>
<xml_diff>
--- a/docs/control-plane/00_MASTER_CONTROL_INDEX.xlsx
+++ b/docs/control-plane/00_MASTER_CONTROL_INDEX.xlsx
@@ -8,15 +8,16 @@
     <sheet sheetId="2" name="CONTROL_MAP" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="NAMING_CONVENTION" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="AI_OPERATING_RULES" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="PLATFORM_MAP" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="MASTER_STATUS" state="visible" r:id="rId9"/>
+    <sheet sheetId="5" name="APPLICATION_TRACKS" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="PLATFORM_MAP" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="MASTER_STATUS" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="325">
   <si>
     <t>00_MASTER_CONTROL_INDEX</t>
   </si>
@@ -690,6 +691,93 @@
     <t>Always resolve: Account -&gt; Environment -&gt; Service -&gt; Resource -&gt; Domain -&gt; Deployment before edits.</t>
   </si>
   <si>
+    <t>Application_ID</t>
+  </si>
+  <si>
+    <t>Application_Name</t>
+  </si>
+  <si>
+    <t>Development_Agent</t>
+  </si>
+  <si>
+    <t>Repository_ID</t>
+  </si>
+  <si>
+    <t>Production_Branch</t>
+  </si>
+  <si>
+    <t>Production_Domain</t>
+  </si>
+  <si>
+    <t>CI_CD_Workflow</t>
+  </si>
+  <si>
+    <t>Deployment_Target</t>
+  </si>
+  <si>
+    <t>Scope_and_Boundaries</t>
+  </si>
+  <si>
+    <t>APP-PUBLIC-WEBSITE</t>
+  </si>
+  <si>
+    <t>Arivahly Public Marketing Website &amp; CMS</t>
+  </si>
+  <si>
+    <t>PUBLIC WEBSITE DEVELOPMENT AGENT</t>
+  </si>
+  <si>
+    <t>REPO-PUBLIC-WEBSITE</t>
+  </si>
+  <si>
+    <t>main</t>
+  </si>
+  <si>
+    <t>arivahly.in</t>
+  </si>
+  <si>
+    <t>.github/workflows/deploy-website.yml (Isolated)</t>
+  </si>
+  <si>
+    <t>Hostinger public_html (Apex Domain Root)</t>
+  </si>
+  <si>
+    <t>Public Website Agent</t>
+  </si>
+  <si>
+    <t>STRICT BOUNDARY: Public marketing pages, CMS, SEO, contact forms, PHP server-rendered site. The ERP Agent MUST NEVER touch or build this project.</t>
+  </si>
+  <si>
+    <t>APP-ONLINE-ERP</t>
+  </si>
+  <si>
+    <t>Arivahly Online Managed Jewellery ERP Platform</t>
+  </si>
+  <si>
+    <t>ERP DEVELOPMENT AGENT</t>
+  </si>
+  <si>
+    <t>REPO-UPSTREAM-MAIN / REPO-HOSTINGER-LIVE</t>
+  </si>
+  <si>
+    <t>feature/production-v1.1.2 / main</t>
+  </si>
+  <si>
+    <t>erp.arivahly.in</t>
+  </si>
+  <si>
+    <t>.github/workflows/production-deploy.yml</t>
+  </si>
+  <si>
+    <t>Hostinger public_html/erp (Subdomain Directory)</t>
+  </si>
+  <si>
+    <t>ERP Development Agent</t>
+  </si>
+  <si>
+    <t>STRICT BOUNDARY: SaaS Admin Panel, CRM, Billing, Ledgers, Portals, Supabase DB/Auth, R2 Vault, Cloudflare WAF, ERP CI/CD. The Public Website Agent MUST NEVER touch this project.</t>
+  </si>
+  <si>
     <t>Component</t>
   </si>
   <si>
@@ -837,6 +925,15 @@
     <t>avs-gold-erp, avs-erp-hostinger-live, avs-erp-baseline-backup</t>
   </si>
   <si>
+    <t>Total Application Tracks</t>
+  </si>
+  <si>
+    <t>00_MASTER_CONTROL_INDEX.xlsx</t>
+  </si>
+  <si>
+    <t>APP-PUBLIC-WEBSITE (arivahly.in) &amp; APP-ONLINE-ERP (erp.arivahly.in)</t>
+  </si>
+  <si>
     <t>Total Domains Configured</t>
   </si>
   <si>
@@ -888,7 +985,7 @@
     <t>Overall Verification Timestamp</t>
   </si>
   <si>
-    <t>2026-09-05T13:20:00+05:30</t>
+    <t>2026-09-05T14:00:00+05:30</t>
   </si>
   <si>
     <t>FINAL_ONLINE_PRODUCTION_AUDIT.md</t>
@@ -2568,6 +2665,124 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="5" max="5" width="36" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
+    <col min="7" max="8" width="51" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="54" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>252</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2589,40 +2804,40 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>224</v>
+        <v>253</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>225</v>
+        <v>254</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>226</v>
+        <v>255</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>227</v>
+        <v>256</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>228</v>
+        <v>257</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>229</v>
+        <v>258</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>230</v>
+        <v>259</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>231</v>
+        <v>260</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>232</v>
+        <v>261</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>233</v>
+        <v>262</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>234</v>
+        <v>263</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>28</v>
@@ -2636,7 +2851,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>235</v>
+        <v>264</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>158</v>
@@ -2654,25 +2869,25 @@
         <v>183</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>236</v>
+        <v>265</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>237</v>
+        <v>266</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>238</v>
+        <v>267</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>239</v>
+        <v>268</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>188</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>240</v>
+        <v>269</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>241</v>
+        <v>270</v>
       </c>
       <c r="N2" s="7" t="s">
         <v>42</v>
@@ -2683,43 +2898,43 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>244</v>
+        <v>273</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>245</v>
+        <v>274</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>246</v>
+        <v>275</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>248</v>
+        <v>277</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>249</v>
+        <v>278</v>
       </c>
       <c r="N3" s="7" t="s">
         <v>42</v>
@@ -2730,43 +2945,43 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>250</v>
+        <v>279</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>251</v>
+        <v>280</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>252</v>
+        <v>281</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>253</v>
+        <v>282</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>254</v>
+        <v>283</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>255</v>
+        <v>284</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>256</v>
+        <v>285</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>257</v>
+        <v>286</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>258</v>
+        <v>287</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>259</v>
+        <v>288</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>260</v>
+        <v>289</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>261</v>
+        <v>290</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>262</v>
+        <v>291</v>
       </c>
       <c r="N4" s="7" t="s">
         <v>42</v>
@@ -2781,9 +2996,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -2794,21 +3009,21 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>263</v>
+        <v>292</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>264</v>
+        <v>293</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>265</v>
+        <v>294</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>266</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>267</v>
+        <v>296</v>
       </c>
       <c r="B2" s="6">
         <v>6</v>
@@ -2817,12 +3032,12 @@
         <v>36</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>268</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>269</v>
+        <v>298</v>
       </c>
       <c r="B3" s="6">
         <v>3</v>
@@ -2831,12 +3046,12 @@
         <v>58</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>270</v>
+        <v>299</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>271</v>
+        <v>300</v>
       </c>
       <c r="B4" s="6">
         <v>3</v>
@@ -2845,119 +3060,133 @@
         <v>75</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="B5" s="6">
         <v>2</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>92</v>
+        <v>303</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>274</v>
+        <v>304</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="B6" s="6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>276</v>
+        <v>306</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>277</v>
+        <v>307</v>
       </c>
       <c r="B7" s="6">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>116</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>278</v>
+        <v>308</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>279</v>
+        <v>309</v>
       </c>
       <c r="B8" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>280</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>281</v>
+        <v>311</v>
       </c>
       <c r="B9" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>282</v>
+        <v>137</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>283</v>
+        <v>312</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>284</v>
+        <v>313</v>
       </c>
       <c r="B10" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>116</v>
+        <v>314</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>285</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>287</v>
+        <v>316</v>
+      </c>
+      <c r="B11" s="6">
+        <v>1</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>288</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>289</v>
+        <v>318</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>290</v>
+        <v>319</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>291</v>
+        <v>92</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>292</v>
+        <v>320</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>324</v>
       </c>
     </row>
   </sheetData>

</xml_diff>